<commit_message>
feat: add achievement system and baram calendar
</commit_message>
<xml_diff>
--- a/resources/table/achievement.xlsx
+++ b/resources/table/achievement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA29110-4E48-4D46-A6EA-C9F4888D2691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A55B08F3-00E3-405A-BF13-12EFB5605B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{51E714AE-D231-4317-A66B-833316D0EFD8}"/>
   </bookViews>
@@ -1241,7 +1241,8 @@
   <cols>
     <col min="1" max="1" width="7.25" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="9.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -1295,7 +1296,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="2">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>

</xml_diff>